<commit_message>
Modified F414 thrust & new F18E file
</commit_message>
<xml_diff>
--- a/Sizing/Lookups/engine_lookup.xlsx
+++ b/Sizing/Lookups/engine_lookup.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roymw\OneDrive - Virginia Tech\Documents\AOE assigments folder\MATLAB\Matlab courses\Air Vehicle Design\Repository\team10aiaa\Sizing\Lookups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01E765BE-F16D-4522-8316-3648A523C18A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8265B00F-AFD6-45D7-8A36-D5ACA3F619BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -386,14 +386,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.5546875" customWidth="1"/>
-    <col min="2" max="2" width="25.5546875" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" customWidth="1"/>
+    <col min="1" max="1" width="14.54296875" customWidth="1"/>
+    <col min="2" max="2" width="25.54296875" customWidth="1"/>
+    <col min="3" max="3" width="23.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -419,7 +419,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -445,7 +445,7 @@
         <v>45000000</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -471,15 +471,15 @@
         <v>45000000</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>57800</v>
+        <v>61932.589336800003</v>
       </c>
       <c r="C4">
-        <v>97900</v>
+        <v>92207.185546399996</v>
       </c>
       <c r="D4">
         <v>30</v>
@@ -497,7 +497,7 @@
         <v>45000000</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -523,7 +523,7 @@
         <v>45000000</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -549,7 +549,7 @@
         <v>45000000</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
Built three functions to enable calculation of component weights using Raymer estimations. Moved some files around to clean up the Sizing folder
</commit_message>
<xml_diff>
--- a/Sizing/Lookups/engine_lookup.xlsx
+++ b/Sizing/Lookups/engine_lookup.xlsx
@@ -5,27 +5,38 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roymw\OneDrive - Virginia Tech\Documents\AOE assigments folder\MATLAB\Matlab courses\Air Vehicle Design\Repository\team10aiaa\Sizing\Lookups\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\Lookups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8265B00F-AFD6-45D7-8A36-D5ACA3F619BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{824F1BEA-FF47-4BD0-882A-9CADFE6BB3C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>F404</t>
   </si>
@@ -67,6 +78,12 @@
   </si>
   <si>
     <t>H20</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>diameter</t>
   </si>
 </sst>
 </file>
@@ -385,15 +402,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.54296875" customWidth="1"/>
-    <col min="2" max="2" width="25.54296875" customWidth="1"/>
-    <col min="3" max="3" width="23.453125" customWidth="1"/>
+    <col min="1" max="1" width="14.5546875" customWidth="1"/>
+    <col min="2" max="2" width="25.5546875" customWidth="1"/>
+    <col min="3" max="3" width="23.44140625" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" customWidth="1"/>
+    <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -418,8 +437,14 @@
       <c r="H1" t="s">
         <v>11</v>
       </c>
+      <c r="I1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -444,8 +469,15 @@
       <c r="H2" s="1">
         <v>45000000</v>
       </c>
+      <c r="I2">
+        <f>1035*9.805</f>
+        <v>10148.174999999999</v>
+      </c>
+      <c r="J2">
+        <v>0.89</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -470,8 +502,15 @@
       <c r="H3" s="1">
         <v>45000000</v>
       </c>
+      <c r="I3">
+        <f>2910*9.805</f>
+        <v>28532.55</v>
+      </c>
+      <c r="J3">
+        <v>1.17</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -496,8 +535,15 @@
       <c r="H4" s="1">
         <v>45000000</v>
       </c>
+      <c r="I4">
+        <f>1110*9.805</f>
+        <v>10883.55</v>
+      </c>
+      <c r="J4">
+        <v>0.89</v>
+      </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -522,8 +568,15 @@
       <c r="H5" s="1">
         <v>45000000</v>
       </c>
+      <c r="I5">
+        <f>1377*9.805</f>
+        <v>13501.484999999999</v>
+      </c>
+      <c r="J5">
+        <v>0.88</v>
+      </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -548,8 +601,15 @@
       <c r="H6" s="1">
         <v>45000000</v>
       </c>
+      <c r="I6">
+        <f>1740*9.805</f>
+        <v>17060.7</v>
+      </c>
+      <c r="J6">
+        <v>0.90600000000000003</v>
+      </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -573,6 +633,13 @@
       </c>
       <c r="H7" s="1">
         <v>45000000</v>
+      </c>
+      <c r="I7">
+        <f>1.65*9.805</f>
+        <v>16.178249999999998</v>
+      </c>
+      <c r="J7">
+        <v>0.111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>